<commit_message>
situacioni edit baloni file 2010
</commit_message>
<xml_diff>
--- a/Legalizim/1-Situacioni/regjistri/18-Koordinatat-e-ndërtesës-700-64-Verimi-Bibaj-Legalizim.xlsx
+++ b/Legalizim/1-Situacioni/regjistri/18-Koordinatat-e-ndërtesës-700-64-Verimi-Bibaj-Legalizim.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\valon\OneDrive\Desktop\puna\Ferizaj\ferizaj\87-3-Verimi-Bibaj\700-64-Verimi-Bibja-Legalizim\1-Situacioni\regjistri\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\valon\OneDrive\Desktop\puna\Ferizaj\ferizaj\87-3-Verimi-Bibaj\Legalizim\1-Situacioni\regjistri\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="23" documentId="13_ncr:1_{958F09B9-7E06-41D6-BE73-5E7FF4D31BC3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{2FC3C8BC-6845-4A60-801E-BE8AB8A121E6}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE505ED9-4881-4EBE-8567-7F24A592B178}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="528" yWindow="336" windowWidth="28272" windowHeight="15876" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="528" yWindow="336" windowWidth="28272" windowHeight="15876" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2148,7 +2148,7 @@
       <c r="J19" s="4"/>
       <c r="K19" s="4"/>
     </row>
-    <row r="20" spans="1:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:11" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A20" s="4"/>
       <c r="B20" s="4"/>
       <c r="C20" s="11">

</xml_diff>